<commit_message>
chore: update Shams CRM accounts
</commit_message>
<xml_diff>
--- a/src/lib/shams-crm/agent-workbook.xlsx
+++ b/src/lib/shams-crm/agent-workbook.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="34">
   <si>
     <t>milaportal_email</t>
   </si>
@@ -112,6 +112,15 @@
   </si>
   <si>
     <t>kamr</t>
+  </si>
+  <si>
+    <t>Ahmed Abdelsalam</t>
+  </si>
+  <si>
+    <t>ahmed.deyaa@milaserv.com</t>
+  </si>
+  <si>
+    <t>Ahmed</t>
   </si>
 </sst>
 </file>
@@ -164,12 +173,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -451,7 +461,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29.5" customWidth="1"/>
@@ -629,14 +639,35 @@
         <v>0</v>
       </c>
     </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D9">
+        <v>4007</v>
+      </c>
+      <c r="E9" t="s">
+        <v>33</v>
+      </c>
+      <c r="F9">
+        <v>123</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
     <hyperlink ref="A3" r:id="rId2"/>
     <hyperlink ref="A4" r:id="rId3"/>
     <hyperlink ref="A8" r:id="rId4"/>
+    <hyperlink ref="A9" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId5"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId6"/>
 </worksheet>
 </file>
</xml_diff>